<commit_message>
Add Stanton landing-zone spaceports to the station seed
Adds the four planetside city spaceports — Riker Memorial (Lorville,
Hurston), Teasa (Orison, Crusader), August Dunlow (Area18, ArcCorp),
and New Babbage Interstellar (New Babbage, microTech). station_type
'spaceport'; each sort_order slots just after its city's
major_location. Station seed is now 295.

Voice-handoff spreadsheet regenerated to include them.

Note: starcitizen.tools was returning HTTP 503 so the category page
could not be scraped — these four are the complete set of Stanton
city spaceports from game knowledge. If the wiki category lists
others (e.g. in Pyro), they can be appended the same way.
</commit_message>
<xml_diff>
--- a/scm_stations_voice_handoff.xlsx
+++ b/scm_stations_voice_handoff.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G292"/>
+  <dimension ref="A1:G296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1234,17 +1234,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>ArcCorp</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Awala</t>
+          <t>August Dunlow Spaceport</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>spaceport</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -1261,27 +1261,23 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ArcCorp</t>
+          <t>Cellin</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Baijini Point</t>
+          <t>Awala</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>orbital</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E31" t="n">
         <v>0</v>
       </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Bajini; Bageeni; Begini; Magini; Vijini; Baijini</t>
-        </is>
-      </c>
+      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
     </row>
     <row r="32">
@@ -1292,23 +1288,27 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>ArcCorp</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Barton Flats Aid Shelter</t>
+          <t>Baijini Point</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>shelter</t>
+          <t>orbital</t>
         </is>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
-      <c r="F32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Bajini; Bageeni; Begini; Magini; Vijini; Baijini</t>
+        </is>
+      </c>
       <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
@@ -1319,27 +1319,23 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CRU-L5</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Beautiful Glen</t>
+          <t>Barton Flats Aid Shelter</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>lagrange</t>
+          <t>shelter</t>
         </is>
       </c>
       <c r="E33" t="n">
         <v>0</v>
       </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>CRU-L5 Beautiful Glen Station</t>
-        </is>
-      </c>
+      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
@@ -1350,23 +1346,27 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Yela</t>
+          <t>CRU-L5</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Benson Mining Outpost</t>
+          <t>Beautiful Glen</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>outpost</t>
+          <t>lagrange</t>
         </is>
       </c>
       <c r="E34" t="n">
         <v>0</v>
       </c>
-      <c r="F34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>CRU-L5 Beautiful Glen Station</t>
+        </is>
+      </c>
       <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
@@ -1377,17 +1377,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>Yela</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Birbari</t>
+          <t>Benson Mining Outpost</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>outpost</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -1404,17 +1404,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>Cellin</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Boondoggle</t>
+          <t>Birbari</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>forward_operating_base</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -1431,17 +1431,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Bountiful Harvest Hydroponics</t>
+          <t>Boondoggle</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>farm</t>
+          <t>forward_operating_base</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -1463,12 +1463,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Brio's Breaker Yard</t>
+          <t>Bountiful Harvest Hydroponics</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>salvage_yard</t>
+          <t>farm</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -1485,17 +1485,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Broken Patch</t>
+          <t>Brio's Breaker Yard</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>forward_operating_base</t>
+          <t>salvage_yard</t>
         </is>
       </c>
       <c r="E39" t="n">
@@ -1512,17 +1512,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Lyria</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Buckets</t>
+          <t>Broken Patch</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forward_operating_base</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -1539,17 +1539,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Euterpe</t>
+          <t>Lyria</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Bud's Growery</t>
+          <t>Buckets</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>farm</t>
+          <t>other</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -1566,17 +1566,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>microTech</t>
+          <t>Euterpe</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Calhoun Pass Emergency Shelter</t>
+          <t>Bud's Growery</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>emergency_shelter</t>
+          <t>farm</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -1593,17 +1593,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>microTech</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Chilad</t>
+          <t>Calhoun Pass Emergency Shelter</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>emergency_shelter</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -1620,17 +1620,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>microTech</t>
+          <t>Cellin</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Clear View Emergency Shelter</t>
+          <t>Chilad</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>emergency_shelter</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -1647,17 +1647,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Crusader</t>
+          <t>microTech</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Cloudrest Retreat</t>
+          <t>Clear View Emergency Shelter</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>floating_platform_community</t>
+          <t>emergency_shelter</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -1674,17 +1674,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Ita</t>
+          <t>Crusader</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Comm Array ST1-02</t>
+          <t>Cloudrest Retreat</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>comm_array</t>
+          <t>floating_platform_community</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -1701,12 +1701,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>Ita</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Comm Array ST2-28</t>
+          <t>Comm Array ST1-02</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1728,12 +1728,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>Cellin</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Comm Array ST2-47</t>
+          <t>Comm Array ST2-28</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1755,12 +1755,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Yela</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Comm Array ST2-76</t>
+          <t>Comm Array ST2-47</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1782,12 +1782,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Arial</t>
+          <t>Yela</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>CommArray ST1-13</t>
+          <t>Comm Array ST2-76</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1809,12 +1809,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Magda</t>
+          <t>Arial</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>CommArray ST1-48</t>
+          <t>CommArray ST1-13</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1836,12 +1836,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>Magda</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>CommArray ST1-92</t>
+          <t>CommArray ST1-48</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1863,12 +1863,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Lyria</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>CommArray ST3-18</t>
+          <t>CommArray ST1-92</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1890,12 +1890,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Wala</t>
+          <t>Lyria</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>CommArray ST3-35</t>
+          <t>CommArray ST3-18</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1917,12 +1917,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Calliope</t>
+          <t>Wala</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>CommArray ST4-31</t>
+          <t>CommArray ST3-35</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1944,12 +1944,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Clio</t>
+          <t>Calliope</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>CommArray ST4-59</t>
+          <t>CommArray ST4-31</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1971,12 +1971,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Euterpe</t>
+          <t>Clio</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>CommArray ST4-64</t>
+          <t>CommArray ST4-59</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1998,17 +1998,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Yela</t>
+          <t>Euterpe</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Connor's</t>
+          <t>CommArray ST4-64</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>underground_bunker</t>
+          <t>comm_array</t>
         </is>
       </c>
       <c r="E58" t="n">
@@ -2025,17 +2025,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>Yela</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Consumption</t>
+          <t>Connor's</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>forward_operating_base</t>
+          <t>underground_bunker</t>
         </is>
       </c>
       <c r="E59" t="n">
@@ -2052,17 +2052,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>Cellin</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Covalex Distribution Centre S1DC06</t>
+          <t>Consumption</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>distribution_centre</t>
+          <t>forward_operating_base</t>
         </is>
       </c>
       <c r="E60" t="n">
@@ -2079,12 +2079,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>microTech</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Covalex Distribution Centre S4DC05</t>
+          <t>Covalex Distribution Centre S1DC06</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2106,17 +2106,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>microTech</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Covalex Hub Gundo</t>
+          <t>Covalex Distribution Centre S4DC05</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>artificial_satellite</t>
+          <t>distribution_centre</t>
         </is>
       </c>
       <c r="E62" t="n">
@@ -2133,17 +2133,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Arial</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Coven</t>
+          <t>Covalex Hub Gundo</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>forward_operating_base</t>
+          <t>artificial_satellite</t>
         </is>
       </c>
       <c r="E63" t="n">
@@ -2160,17 +2160,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>Arial</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Criska</t>
+          <t>Coven</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>forward_operating_base</t>
         </is>
       </c>
       <c r="E64" t="n">
@@ -2187,17 +2187,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>microTech</t>
+          <t>Cellin</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Cry-Astro Processing Plant 19-02</t>
+          <t>Criska</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>distribution_centre</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E65" t="n">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Cry-Astro Processing Plant 34-12</t>
+          <t>Cry-Astro Processing Plant 19-02</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2241,17 +2241,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>microTech</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Cutter's Rig</t>
+          <t>Cry-Astro Processing Plant 34-12</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>settlement</t>
+          <t>distribution_centre</t>
         </is>
       </c>
       <c r="E67" t="n">
@@ -2268,17 +2268,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Dawu</t>
+          <t>Cutter's Rig</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>settlement</t>
         </is>
       </c>
       <c r="E68" t="n">
@@ -2295,17 +2295,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Yela</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Deakins Research Outpost</t>
+          <t>Dawu</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>research_outpost</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E69" t="n">
@@ -2322,17 +2322,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Euterpe</t>
+          <t>Yela</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Devlin Scrap &amp; Salvage</t>
+          <t>Deakins Research Outpost</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>salvage_yard</t>
+          <t>research_outpost</t>
         </is>
       </c>
       <c r="E70" t="n">
@@ -2349,17 +2349,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>Euterpe</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Dipur</t>
+          <t>Devlin Scrap &amp; Salvage</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>salvage_yard</t>
         </is>
       </c>
       <c r="E71" t="n">
@@ -2376,17 +2376,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>Cellin</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Dunlow Ridge</t>
+          <t>Dipur</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>shelter</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E72" t="n">
@@ -2403,17 +2403,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Dupree Industrial Manufacturing Facility</t>
+          <t>Dunlow Ridge</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>distribution_centre</t>
+          <t>shelter</t>
         </is>
       </c>
       <c r="E73" t="n">
@@ -2430,17 +2430,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Eager Flats</t>
+          <t>Dupree Industrial Manufacturing Facility</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>shelter</t>
+          <t>distribution_centre</t>
         </is>
       </c>
       <c r="E74" t="n">
@@ -2457,17 +2457,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Crusader</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Empyrean Park</t>
+          <t>Eager Flats</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>floating_platform_community</t>
+          <t>shelter</t>
         </is>
       </c>
       <c r="E75" t="n">
@@ -2484,17 +2484,17 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>Crusader</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Erden</t>
+          <t>Empyrean Park</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>floating_platform_community</t>
         </is>
       </c>
       <c r="E76" t="n">
@@ -2511,27 +2511,23 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Everus Harbor</t>
+          <t>Erden</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>orbital</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E77" t="n">
         <v>0</v>
       </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>Everest Harbor; Evers Harbor; Evers; Everus</t>
-        </is>
-      </c>
+      <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
     </row>
     <row r="78">
@@ -2542,23 +2538,27 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Fetch</t>
+          <t>Everus Harbor</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>forward_operating_base</t>
+          <t>orbital</t>
         </is>
       </c>
       <c r="E78" t="n">
         <v>0</v>
       </c>
-      <c r="F78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Everest Harbor; Evers Harbor; Evers; Everus</t>
+        </is>
+      </c>
       <c r="G78" t="inlineStr"/>
     </row>
     <row r="79">
@@ -2569,17 +2569,17 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>Cellin</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Finn's Folly</t>
+          <t>Fetch</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>settlement</t>
+          <t>forward_operating_base</t>
         </is>
       </c>
       <c r="E79" t="n">
@@ -2596,17 +2596,17 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Flanagan's Ravine</t>
+          <t>Finn's Folly</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>shelter</t>
+          <t>settlement</t>
         </is>
       </c>
       <c r="E80" t="n">
@@ -2628,12 +2628,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Gallete Family Farms</t>
+          <t>Flanagan's Ravine</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>outpost</t>
+          <t>shelter</t>
         </is>
       </c>
       <c r="E81" t="n">
@@ -2655,12 +2655,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Gandan</t>
+          <t>Gallete Family Farms</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>outpost</t>
         </is>
       </c>
       <c r="E82" t="n">
@@ -2677,17 +2677,17 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>microTech</t>
+          <t>Cellin</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Ghost Hollow</t>
+          <t>Gandan</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>settlement</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E83" t="n">
@@ -2704,17 +2704,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Magda</t>
+          <t>microTech</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Gonzo</t>
+          <t>Ghost Hollow</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>forward_operating_base</t>
+          <t>settlement</t>
         </is>
       </c>
       <c r="E84" t="n">
@@ -2731,17 +2731,17 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>Magda</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Greycat Stanton I Production Complex-B</t>
+          <t>Gonzo</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>distribution_centre</t>
+          <t>forward_operating_base</t>
         </is>
       </c>
       <c r="E85" t="n">
@@ -2758,12 +2758,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>microTech</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Greycat Stanton IV Production Complex-A</t>
+          <t>Greycat Stanton I Production Complex-B</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2785,17 +2785,17 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Yela</t>
+          <t>microTech</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>GrimHEX</t>
+          <t>Greycat Stanton IV Production Complex-A</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>artificial_satellite</t>
+          <t>distribution_centre</t>
         </is>
       </c>
       <c r="E87" t="n">
@@ -2817,12 +2817,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Half Stack</t>
+          <t>GrimHEX</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>forward_operating_base</t>
+          <t>artificial_satellite</t>
         </is>
       </c>
       <c r="E88" t="n">
@@ -2844,12 +2844,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Hasik</t>
+          <t>Half Stack</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>forward_operating_base</t>
         </is>
       </c>
       <c r="E89" t="n">
@@ -2866,17 +2866,17 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>Yela</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>HDMS-Anderson</t>
+          <t>Hasik</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>mining_outpost</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E90" t="n">
@@ -2893,12 +2893,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Arial</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>HDMS-Bezdek</t>
+          <t>HDMS-Anderson</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2920,12 +2920,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>Arial</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>HDMS-Edmond</t>
+          <t>HDMS-Bezdek</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2952,7 +2952,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>HDMS-Hadley</t>
+          <t>HDMS-Edmond</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -2974,12 +2974,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Magda</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>HDMS-Hahn</t>
+          <t>HDMS-Hadley</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -3001,12 +3001,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Arial</t>
+          <t>Magda</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>HDMS-Lathan</t>
+          <t>HDMS-Hahn</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -3028,12 +3028,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>Arial</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>HDMS-Norgaard</t>
+          <t>HDMS-Lathan</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -3055,12 +3055,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>HDMS-Oparei</t>
+          <t>HDMS-Norgaard</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -3082,12 +3082,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Magda</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>HDMS-Perlman</t>
+          <t>HDMS-Oparei</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -3109,12 +3109,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>Magda</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>HDMS-Pinewood</t>
+          <t>HDMS-Perlman</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -3136,12 +3136,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Ita</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>HDMS-Ryder</t>
+          <t>HDMS-Pinewood</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -3163,12 +3163,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>Ita</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>HDMS-Stanhope</t>
+          <t>HDMS-Ryder</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -3195,7 +3195,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>HDMS-Thedus</t>
+          <t>HDMS-Stanhope</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -3217,12 +3217,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Ita</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>HDMS-Woodruff</t>
+          <t>HDMS-Thedus</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -3244,17 +3244,17 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>Ita</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>HDPC-Cassillo</t>
+          <t>HDMS-Woodruff</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>distribution_centre</t>
+          <t>mining_outpost</t>
         </is>
       </c>
       <c r="E104" t="n">
@@ -3276,7 +3276,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>HDPC-Farnesway</t>
+          <t>HDPC-Cassillo</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -3303,12 +3303,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>HDRSO-Baier</t>
+          <t>HDPC-Farnesway</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>distribution_centre</t>
         </is>
       </c>
       <c r="E106" t="n">
@@ -3330,7 +3330,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>HDRSO-Bardie</t>
+          <t>HDRSO-Baier</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3357,7 +3357,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>HDRSO-Bersch</t>
+          <t>HDRSO-Bardie</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -3384,7 +3384,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>HDRSO-Bowes</t>
+          <t>HDRSO-Bersch</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3411,7 +3411,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>HDRSO-Bramen</t>
+          <t>HDRSO-Bowes</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3438,7 +3438,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>HDRSO-Brel</t>
+          <t>HDRSO-Bramen</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -3465,7 +3465,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>HDRSO-Cronshaw</t>
+          <t>HDRSO-Brel</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -3492,7 +3492,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>HDRSO-Foster</t>
+          <t>HDRSO-Cronshaw</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -3519,7 +3519,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>HDRSO-Franz</t>
+          <t>HDRSO-Foster</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3546,7 +3546,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>HDRSO-Giblin</t>
+          <t>HDRSO-Franz</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -3573,7 +3573,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>HDRSO-Hosley</t>
+          <t>HDRSO-Giblin</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>HDRSO-Malloy</t>
+          <t>HDRSO-Hosley</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -3627,7 +3627,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>HDRSO-Marling</t>
+          <t>HDRSO-Malloy</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>HDRSO-McKuen</t>
+          <t>HDRSO-Marling</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -3681,7 +3681,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>HDRSO-Newman</t>
+          <t>HDRSO-McKuen</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -3708,7 +3708,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>HDRSO-Olliff</t>
+          <t>HDRSO-Newman</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -3735,7 +3735,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>HDRSO-Pearce</t>
+          <t>HDRSO-Olliff</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -3762,7 +3762,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>HDRSO-Sheppard</t>
+          <t>HDRSO-Pearce</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>HDRSO-Sims</t>
+          <t>HDRSO-Sheppard</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -3816,7 +3816,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>HDRSO-Stott</t>
+          <t>HDRSO-Sims</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -3843,7 +3843,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>HDRSO-Tillman</t>
+          <t>HDRSO-Stott</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -3870,7 +3870,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>HDRSO-Walker</t>
+          <t>HDRSO-Tillman</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -3897,7 +3897,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>HDRSO-Wyatt</t>
+          <t>HDRSO-Walker</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -3924,12 +3924,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>HDSF-Adlai</t>
+          <t>HDRSO-Wyatt</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>underground_facility</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E129" t="n">
@@ -3951,7 +3951,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>HDSF-Barnabas</t>
+          <t>HDSF-Adlai</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -3978,7 +3978,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>HDSF-Breckinridge</t>
+          <t>HDSF-Barnabas</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -4005,7 +4005,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>HDSF-Colfax</t>
+          <t>HDSF-Breckinridge</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -4032,7 +4032,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>HDSF-Damaris</t>
+          <t>HDSF-Colfax</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -4059,7 +4059,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>HDSF-Elbridge</t>
+          <t>HDSF-Damaris</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -4086,7 +4086,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>HDSF-Hendricks</t>
+          <t>HDSF-Elbridge</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -4113,7 +4113,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>HDSF-Hiram</t>
+          <t>HDSF-Hendricks</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -4140,7 +4140,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>HDSF-Hobart</t>
+          <t>HDSF-Hiram</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>HDSF-Ishmael</t>
+          <t>HDSF-Hobart</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -4194,7 +4194,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>HDSF-Millerand</t>
+          <t>HDSF-Ishmael</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -4221,12 +4221,12 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>HDSF-Palomar</t>
+          <t>HDSF-Millerand</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>underground_facility</t>
         </is>
       </c>
       <c r="E140" t="n">
@@ -4248,12 +4248,12 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>HDSF-Rufus</t>
+          <t>HDSF-Palomar</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>underground_facility</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E141" t="n">
@@ -4275,7 +4275,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>HDSF-Sherman</t>
+          <t>HDSF-Rufus</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -4302,7 +4302,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>HDSF-Tamar</t>
+          <t>HDSF-Sherman</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -4329,7 +4329,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>HDSF-Tompkins</t>
+          <t>HDSF-Tamar</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -4356,7 +4356,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>HDSF-Zacharias</t>
+          <t>HDSF-Tompkins</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -4378,17 +4378,17 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Hickes Research Outpost</t>
+          <t>HDSF-Zacharias</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>research_outpost</t>
+          <t>underground_facility</t>
         </is>
       </c>
       <c r="E146" t="n">
@@ -4405,17 +4405,17 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>Cellin</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Hospice</t>
+          <t>Hickes Research Outpost</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>forward_operating_base</t>
+          <t>research_outpost</t>
         </is>
       </c>
       <c r="E147" t="n">
@@ -4432,17 +4432,17 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Lyria</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Humboldt Mines</t>
+          <t>Hospice</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>mining_outpost</t>
+          <t>forward_operating_base</t>
         </is>
       </c>
       <c r="E148" t="n">
@@ -4459,17 +4459,17 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Yela</t>
+          <t>Lyria</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Iteke</t>
+          <t>Humboldt Mines</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>mining_outpost</t>
         </is>
       </c>
       <c r="E149" t="n">
@@ -4486,17 +4486,17 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>Yela</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Julep Ravine</t>
+          <t>Iteke</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>shelter</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E150" t="n">
@@ -4513,17 +4513,17 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>Cellin</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Jumptown</t>
+          <t>Julep Ravine</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>drug_lab</t>
+          <t>shelter</t>
         </is>
       </c>
       <c r="E151" t="n">
@@ -4540,17 +4540,17 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Klescher Rehabilitation Facility</t>
+          <t>Jumptown</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>prison</t>
+          <t>drug_lab</t>
         </is>
       </c>
       <c r="E152" t="n">
@@ -4567,17 +4567,17 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Yela</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Klipra</t>
+          <t>Klescher Rehabilitation Facility</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>prison</t>
         </is>
       </c>
       <c r="E153" t="n">
@@ -4599,12 +4599,12 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Kosso Basin Aid Shelter</t>
+          <t>Klipra</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>shelter</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E154" t="n">
@@ -4621,17 +4621,17 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>Yela</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Kota</t>
+          <t>Kosso Basin Aid Shelter</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>shelter</t>
         </is>
       </c>
       <c r="E155" t="n">
@@ -4648,17 +4648,17 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>Cellin</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Kudre Ore</t>
+          <t>Kota</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>outpost</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E156" t="n">
@@ -4680,12 +4680,12 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Lamina OLP</t>
+          <t>Kudre Ore</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>orbital_laser_platform</t>
+          <t>outpost</t>
         </is>
       </c>
       <c r="E157" t="n">
@@ -4707,12 +4707,12 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Lamina PAF-I</t>
+          <t>Lamina OLP</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>planetary_alignment_facility</t>
+          <t>orbital_laser_platform</t>
         </is>
       </c>
       <c r="E158" t="n">
@@ -4734,7 +4734,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Lamina PAF-II</t>
+          <t>Lamina PAF-I</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -4761,7 +4761,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Lamina PAF-III</t>
+          <t>Lamina PAF-II</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -4783,17 +4783,17 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Lyria</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Launch Pad</t>
+          <t>Lamina PAF-III</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>planetary_alignment_facility</t>
         </is>
       </c>
       <c r="E161" t="n">
@@ -4810,17 +4810,17 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>Lyria</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Lespin</t>
+          <t>Launch Pad</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>other</t>
         </is>
       </c>
       <c r="E162" t="n">
@@ -4837,27 +4837,23 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>ARC-L2</t>
+          <t>Cellin</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Lively Pathway</t>
+          <t>Lespin</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>lagrange</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E163" t="n">
         <v>0</v>
       </c>
-      <c r="F163" t="inlineStr">
-        <is>
-          <t>ARC-L2 Lively Pathway Station</t>
-        </is>
-      </c>
+      <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr"/>
     </row>
     <row r="164">
@@ -4868,12 +4864,12 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>MIC-L2</t>
+          <t>ARC-L2</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Long Forest</t>
+          <t>Lively Pathway</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -4886,7 +4882,7 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>MIC-L2 Long Forest Station; Long Force</t>
+          <t>ARC-L2 Lively Pathway Station</t>
         </is>
       </c>
       <c r="G164" t="inlineStr"/>
@@ -4899,23 +4895,27 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>MIC-L2</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Lorville</t>
+          <t>Long Forest</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>major_location</t>
+          <t>lagrange</t>
         </is>
       </c>
       <c r="E165" t="n">
         <v>0</v>
       </c>
-      <c r="F165" t="inlineStr"/>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>MIC-L2 Long Forest Station; Long Force</t>
+        </is>
+      </c>
       <c r="G165" t="inlineStr"/>
     </row>
     <row r="166">
@@ -4926,17 +4926,17 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Lyria</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Loveridge Mineral Reserve</t>
+          <t>Lorville</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>mining_outpost</t>
+          <t>major_location</t>
         </is>
       </c>
       <c r="E166" t="n">
@@ -4953,17 +4953,17 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>Lyria</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Lowdown</t>
+          <t>Loveridge Mineral Reserve</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>forward_operating_base</t>
+          <t>mining_outpost</t>
         </is>
       </c>
       <c r="E167" t="n">
@@ -4985,12 +4985,12 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Ludlow</t>
+          <t>Lowdown</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>settlement</t>
+          <t>forward_operating_base</t>
         </is>
       </c>
       <c r="E168" t="n">
@@ -5007,17 +5007,17 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Yela</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Mainline</t>
+          <t>Ludlow</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>forward_operating_base</t>
+          <t>settlement</t>
         </is>
       </c>
       <c r="E169" t="n">
@@ -5034,17 +5034,17 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>Yela</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Maker's Point</t>
+          <t>Mainline</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>settlement</t>
+          <t>forward_operating_base</t>
         </is>
       </c>
       <c r="E170" t="n">
@@ -5061,17 +5061,17 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Menian</t>
+          <t>Maker's Point</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>settlement</t>
         </is>
       </c>
       <c r="E171" t="n">
@@ -5088,17 +5088,17 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>microTech</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>MicroTech Logistics Depot S4LD01</t>
+          <t>Menian</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>distribution_centre</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E172" t="n">
@@ -5120,7 +5120,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>MicroTech Logistics Depot S4LD13</t>
+          <t>MicroTech Logistics Depot S4LD01</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -5142,17 +5142,17 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Yela</t>
+          <t>microTech</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Miner's Lament</t>
+          <t>MicroTech Logistics Depot S4LD13</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>natural_satellite</t>
+          <t>distribution_centre</t>
         </is>
       </c>
       <c r="E174" t="n">
@@ -5169,17 +5169,17 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>Yela</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Minlo Spire</t>
+          <t>Miner's Lament</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>forward_operating_base</t>
+          <t>natural_satellite</t>
         </is>
       </c>
       <c r="E175" t="n">
@@ -5196,17 +5196,17 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Mogote</t>
+          <t>Minlo Spire</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>shelter</t>
+          <t>forward_operating_base</t>
         </is>
       </c>
       <c r="E176" t="n">
@@ -5223,17 +5223,17 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Yela</t>
+          <t>Cellin</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Moka</t>
+          <t>Mogote</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>shelter</t>
         </is>
       </c>
       <c r="E177" t="n">
@@ -5250,12 +5250,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>Yela</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Moluto</t>
+          <t>Moka</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -5277,17 +5277,17 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>microTech</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>MT DataCenter 2UB-RB9-5</t>
+          <t>Moluto</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>data_center</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E179" t="n">
@@ -5309,7 +5309,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>MT DataCenter 4HJ-LVE-A</t>
+          <t>MT DataCenter 2UB-RB9-5</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -5336,7 +5336,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>MT DataCenter 5WQ-R2V-C</t>
+          <t>MT DataCenter 4HJ-LVE-A</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>MT DataCenter 8FK-Q2X-K</t>
+          <t>MT DataCenter 5WQ-R2V-C</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -5390,7 +5390,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>MT DataCenter D79-ECG-R</t>
+          <t>MT DataCenter 8FK-Q2X-K</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -5417,7 +5417,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>MT DataCenter E2Q-NSG-Y</t>
+          <t>MT DataCenter D79-ECG-R</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -5444,7 +5444,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>MT DataCenter L8P-JUC-8</t>
+          <t>MT DataCenter E2Q-NSG-Y</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -5471,7 +5471,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>MT DataCenter QVX-J88-J</t>
+          <t>MT DataCenter L8P-JUC-8</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -5498,7 +5498,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>MT DataCenter TMG-XEV-2</t>
+          <t>MT DataCenter QVX-J88-J</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -5525,12 +5525,12 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>MT OpCenter LTI-4</t>
+          <t>MT DataCenter TMG-XEV-2</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>opcenter</t>
+          <t>data_center</t>
         </is>
       </c>
       <c r="E188" t="n">
@@ -5547,17 +5547,17 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Yela</t>
+          <t>microTech</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Nakamura Valley Aid Shelter</t>
+          <t>MT OpCenter LTI-4</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>shelter</t>
+          <t>opcenter</t>
         </is>
       </c>
       <c r="E189" t="n">
@@ -5574,17 +5574,17 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Magda</t>
+          <t>Yela</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Nevermind</t>
+          <t>Nakamura Valley Aid Shelter</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>forward_operating_base</t>
+          <t>shelter</t>
         </is>
       </c>
       <c r="E190" t="n">
@@ -5601,17 +5601,17 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>microTech</t>
+          <t>Magda</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>New Babbage</t>
+          <t>Nevermind</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>major_location</t>
+          <t>forward_operating_base</t>
         </is>
       </c>
       <c r="E191" t="n">
@@ -5628,17 +5628,17 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>microTech</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>NT-999-XV</t>
+          <t>New Babbage</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>underground_bunker</t>
+          <t>major_location</t>
         </is>
       </c>
       <c r="E192" t="n">
@@ -5655,17 +5655,17 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>microTech</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>NT-999-XVI</t>
+          <t>New Babbage Interstellar Spaceport</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>underground_bunker</t>
+          <t>spaceport</t>
         </is>
       </c>
       <c r="E193" t="n">
@@ -5682,17 +5682,17 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Yela</t>
+          <t>Cellin</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>NT-999-XX</t>
+          <t>NT-999-XV</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>outpost</t>
+          <t>underground_bunker</t>
         </is>
       </c>
       <c r="E194" t="n">
@@ -5709,12 +5709,12 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Yela</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>NT-999-XXII</t>
+          <t>NT-999-XVI</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -5736,12 +5736,12 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>Yela</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Nuen Waste Management</t>
+          <t>NT-999-XX</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -5763,17 +5763,17 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>microTech</t>
+          <t>Yela</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Nuiqsut Emergency Shelter</t>
+          <t>NT-999-XXII</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>emergency_shelter</t>
+          <t>underground_bunker</t>
         </is>
       </c>
       <c r="E197" t="n">
@@ -5790,17 +5790,17 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Yela</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Opal</t>
+          <t>Nuen Waste Management</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>outpost</t>
         </is>
       </c>
       <c r="E198" t="n">
@@ -5817,17 +5817,17 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Crusader</t>
+          <t>microTech</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Orison</t>
+          <t>Nuiqsut Emergency Shelter</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>major_location</t>
+          <t>emergency_shelter</t>
         </is>
       </c>
       <c r="E199" t="n">
@@ -5844,12 +5844,12 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>Yela</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Pakote</t>
+          <t>Opal</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -5871,17 +5871,17 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Yela</t>
+          <t>Crusader</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Peska</t>
+          <t>Orison</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>major_location</t>
         </is>
       </c>
       <c r="E201" t="n">
@@ -5898,17 +5898,17 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>Cellin</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Picker's Field</t>
+          <t>Pakote</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>settlement</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E202" t="n">
@@ -5925,17 +5925,17 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>microTech</t>
+          <t>Yela</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Point Wain Emergency Shelter</t>
+          <t>Peska</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>emergency_shelter</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E203" t="n">
@@ -5952,27 +5952,23 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>microTech</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Port Tressler</t>
+          <t>Picker's Field</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>orbital</t>
+          <t>settlement</t>
         </is>
       </c>
       <c r="E204" t="n">
         <v>0</v>
       </c>
-      <c r="F204" t="inlineStr">
-        <is>
-          <t>Tressler; Point Tressler</t>
-        </is>
-      </c>
+      <c r="F204" t="inlineStr"/>
       <c r="G204" t="inlineStr"/>
     </row>
     <row r="205">
@@ -5983,17 +5979,17 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>microTech</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Prashad</t>
+          <t>Point Wain Emergency Shelter</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>emergency_shelter</t>
         </is>
       </c>
       <c r="E205" t="n">
@@ -6010,23 +6006,27 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>microTech</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>PRIVATE PROPERTY</t>
+          <t>Port Tressler</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>outpost</t>
+          <t>orbital</t>
         </is>
       </c>
       <c r="E206" t="n">
         <v>0</v>
       </c>
-      <c r="F206" t="inlineStr"/>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Tressler; Point Tressler</t>
+        </is>
+      </c>
       <c r="G206" t="inlineStr"/>
     </row>
     <row r="207">
@@ -6037,17 +6037,17 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Crusader</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Prospect Point</t>
+          <t>Prashad</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>floating_platform_community</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E207" t="n">
@@ -6062,24 +6062,25 @@
           <t>Stanton</t>
         </is>
       </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Cellin</t>
+        </is>
+      </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Pyro Jump Point</t>
+          <t>PRIVATE PROPERTY</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>gateway</t>
+          <t>outpost</t>
         </is>
       </c>
       <c r="E208" t="n">
-        <v>1</v>
-      </c>
-      <c r="F208" t="inlineStr">
-        <is>
-          <t>Stanton-Pyro Gate (Stanton side); Stanton Gateway</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F208" t="inlineStr"/>
       <c r="G208" t="inlineStr"/>
     </row>
     <row r="209">
@@ -6090,17 +6091,17 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>Crusader</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Rappel</t>
+          <t>Prospect Point</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>settlement</t>
+          <t>floating_platform_community</t>
         </is>
       </c>
       <c r="E209" t="n">
@@ -6115,25 +6116,24 @@
           <t>Stanton</t>
         </is>
       </c>
-      <c r="B210" t="inlineStr">
-        <is>
-          <t>Calliope</t>
-        </is>
-      </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Rayari Anvik Research Outpost</t>
+          <t>Pyro Jump Point</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>research_outpost</t>
+          <t>gateway</t>
         </is>
       </c>
       <c r="E210" t="n">
-        <v>0</v>
-      </c>
-      <c r="F210" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>Stanton-Pyro Gate (Stanton side); Stanton Gateway</t>
+        </is>
+      </c>
       <c r="G210" t="inlineStr"/>
     </row>
     <row r="211">
@@ -6144,17 +6144,17 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Clio</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Rayari Cantwell Research Outpost</t>
+          <t>Rappel</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>research_outpost</t>
+          <t>settlement</t>
         </is>
       </c>
       <c r="E211" t="n">
@@ -6171,12 +6171,12 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>microTech</t>
+          <t>Calliope</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Rayari Deltana Research Outpost</t>
+          <t>Rayari Anvik Research Outpost</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
@@ -6198,12 +6198,12 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Calliope</t>
+          <t>Clio</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Rayari Kaltag Research Outpost</t>
+          <t>Rayari Cantwell Research Outpost</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
@@ -6230,7 +6230,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Rayari Livengood Research Outpost</t>
+          <t>Rayari Deltana Research Outpost</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
@@ -6252,12 +6252,12 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Clio</t>
+          <t>Calliope</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Rayari McGrath Research Outpost</t>
+          <t>Rayari Kaltag Research Outpost</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
@@ -6279,17 +6279,17 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>microTech</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Reawick</t>
+          <t>Rayari Livengood Research Outpost</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>research_outpost</t>
         </is>
       </c>
       <c r="E216" t="n">
@@ -6306,17 +6306,17 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>Clio</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Reclamation &amp; Disposal Orinth</t>
+          <t>Rayari McGrath Research Outpost</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>salvage_yard</t>
+          <t>research_outpost</t>
         </is>
       </c>
       <c r="E217" t="n">
@@ -6333,17 +6333,17 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>Rico's Remains</t>
+          <t>Reawick</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>forward_operating_base</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E218" t="n">
@@ -6360,17 +6360,17 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Yela</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Rolo's Crater</t>
+          <t>Reclamation &amp; Disposal Orinth</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>forward_operating_base</t>
+          <t>salvage_yard</t>
         </is>
       </c>
       <c r="E219" t="n">
@@ -6387,17 +6387,17 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Ruptura OLP</t>
+          <t>Rico's Remains</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>orbital_laser_platform</t>
+          <t>forward_operating_base</t>
         </is>
       </c>
       <c r="E220" t="n">
@@ -6414,17 +6414,17 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>Ruptura PAF-I</t>
+          <t>Riker Memorial Spaceport</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>planetary_alignment_facility</t>
+          <t>spaceport</t>
         </is>
       </c>
       <c r="E221" t="n">
@@ -6441,17 +6441,17 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>Yela</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>Ruptura PAF-II</t>
+          <t>Rolo's Crater</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>planetary_alignment_facility</t>
+          <t>forward_operating_base</t>
         </is>
       </c>
       <c r="E222" t="n">
@@ -6473,12 +6473,12 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>Ruptura PAF-III</t>
+          <t>Ruptura OLP</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>planetary_alignment_facility</t>
+          <t>orbital_laser_platform</t>
         </is>
       </c>
       <c r="E223" t="n">
@@ -6495,17 +6495,17 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>Saktigar</t>
+          <t>Ruptura PAF-I</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>planetary_alignment_facility</t>
         </is>
       </c>
       <c r="E224" t="n">
@@ -6522,17 +6522,17 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>microTech</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>Sakura Sun Goldenrod Workcenter</t>
+          <t>Ruptura PAF-II</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>distribution_centre</t>
+          <t>planetary_alignment_facility</t>
         </is>
       </c>
       <c r="E225" t="n">
@@ -6549,17 +6549,17 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>Sakura Sun Magnolia Workcenter</t>
+          <t>Ruptura PAF-III</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>distribution_centre</t>
+          <t>planetary_alignment_facility</t>
         </is>
       </c>
       <c r="E226" t="n">
@@ -6576,17 +6576,17 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Wala</t>
+          <t>Cellin</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Samson &amp; Sons Salvage Center</t>
+          <t>Saktigar</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>salvage_yard</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E227" t="n">
@@ -6603,17 +6603,17 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>Lyria</t>
+          <t>microTech</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>Security Depot Lyria-1</t>
+          <t>Sakura Sun Goldenrod Workcenter</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>distribution_centre</t>
         </is>
       </c>
       <c r="E228" t="n">
@@ -6630,17 +6630,17 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>Security Post Kareah</t>
+          <t>Sakura Sun Magnolia Workcenter</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>distribution_centre</t>
         </is>
       </c>
       <c r="E229" t="n">
@@ -6657,27 +6657,23 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Crusader</t>
+          <t>Wala</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>Seraphim Station</t>
+          <t>Samson &amp; Sons Salvage Center</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>orbital</t>
+          <t>salvage_yard</t>
         </is>
       </c>
       <c r="E230" t="n">
         <v>0</v>
       </c>
-      <c r="F230" t="inlineStr">
-        <is>
-          <t>Seraphim</t>
-        </is>
-      </c>
+      <c r="F230" t="inlineStr"/>
       <c r="G230" t="inlineStr"/>
     </row>
     <row r="231">
@@ -6688,17 +6684,17 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Wala</t>
+          <t>Lyria</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>Shady Glen Farms</t>
+          <t>Security Depot Lyria-1</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>farm</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E231" t="n">
@@ -6715,27 +6711,23 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>CRU-L4</t>
+          <t>Cellin</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Shallow Fields</t>
+          <t>Security Post Kareah</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>lagrange</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E232" t="n">
         <v>0</v>
       </c>
-      <c r="F232" t="inlineStr">
-        <is>
-          <t>Shallow Field; Shallow Fields Station</t>
-        </is>
-      </c>
+      <c r="F232" t="inlineStr"/>
       <c r="G232" t="inlineStr"/>
     </row>
     <row r="233">
@@ -6746,17 +6738,17 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>HUR-L1</t>
+          <t>Crusader</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Shallow Frontier</t>
+          <t>Seraphim Station</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>lagrange</t>
+          <t>orbital</t>
         </is>
       </c>
       <c r="E233" t="n">
@@ -6764,7 +6756,7 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>Shallow Frontier Station</t>
+          <t>Seraphim</t>
         </is>
       </c>
       <c r="G233" t="inlineStr"/>
@@ -6777,17 +6769,17 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>Wala</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Sharga</t>
+          <t>Shady Glen Farms</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>farm</t>
         </is>
       </c>
       <c r="E234" t="n">
@@ -6804,23 +6796,27 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Lyria</t>
+          <t>CRU-L4</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Shubin Mining Facility SAL-2</t>
+          <t>Shallow Fields</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>mining_outpost</t>
+          <t>lagrange</t>
         </is>
       </c>
       <c r="E235" t="n">
         <v>0</v>
       </c>
-      <c r="F235" t="inlineStr"/>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>Shallow Field; Shallow Fields Station</t>
+        </is>
+      </c>
       <c r="G235" t="inlineStr"/>
     </row>
     <row r="236">
@@ -6831,23 +6827,27 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Lyria</t>
+          <t>HUR-L1</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>Shubin Mining Facility SAL-5</t>
+          <t>Shallow Frontier</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>mining_outpost</t>
+          <t>lagrange</t>
         </is>
       </c>
       <c r="E236" t="n">
         <v>0</v>
       </c>
-      <c r="F236" t="inlineStr"/>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>Shallow Frontier Station</t>
+        </is>
+      </c>
       <c r="G236" t="inlineStr"/>
     </row>
     <row r="237">
@@ -6858,17 +6858,17 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>Cellin</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>Shubin Mining Facility SCD-1</t>
+          <t>Sharga</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>mining_outpost</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E237" t="n">
@@ -6885,12 +6885,12 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>microTech</t>
+          <t>Lyria</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Shubin Mining Facility SM0-10</t>
+          <t>Shubin Mining Facility SAL-2</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
@@ -6912,12 +6912,12 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>microTech</t>
+          <t>Lyria</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Shubin Mining Facility SM0-13</t>
+          <t>Shubin Mining Facility SAL-5</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
@@ -6939,12 +6939,12 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>microTech</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Shubin Mining Facility SM0-18</t>
+          <t>Shubin Mining Facility SCD-1</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
@@ -6971,7 +6971,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Shubin Mining Facility SM0-22</t>
+          <t>Shubin Mining Facility SM0-10</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
@@ -6993,12 +6993,12 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Calliope</t>
+          <t>microTech</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Shubin Mining Facility SMCa-6</t>
+          <t>Shubin Mining Facility SM0-13</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
@@ -7020,12 +7020,12 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Calliope</t>
+          <t>microTech</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Shubin Mining Facility SMCa-8</t>
+          <t>Shubin Mining Facility SM0-18</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
@@ -7047,17 +7047,17 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Lyria</t>
+          <t>microTech</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Shubin Processing Facility SPAL-12</t>
+          <t>Shubin Mining Facility SM0-22</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>processing_facility</t>
+          <t>mining_outpost</t>
         </is>
       </c>
       <c r="E244" t="n">
@@ -7074,17 +7074,17 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Lyria</t>
+          <t>Calliope</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Shubin Processing Facility SPAL-16</t>
+          <t>Shubin Mining Facility SMCa-6</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>processing_facility</t>
+          <t>mining_outpost</t>
         </is>
       </c>
       <c r="E245" t="n">
@@ -7101,17 +7101,17 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Lyria</t>
+          <t>Calliope</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Shubin Processing Facility SPAL-21</t>
+          <t>Shubin Mining Facility SMCa-8</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>processing_facility</t>
+          <t>mining_outpost</t>
         </is>
       </c>
       <c r="E246" t="n">
@@ -7133,7 +7133,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Shubin Processing Facility SPAL-3</t>
+          <t>Shubin Processing Facility SPAL-12</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -7160,7 +7160,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Shubin Processing Facility SPAL-7</t>
+          <t>Shubin Processing Facility SPAL-16</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -7187,7 +7187,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Shubin Processing Facility SPAL-9</t>
+          <t>Shubin Processing Facility SPAL-21</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
@@ -7209,12 +7209,12 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Calliope</t>
+          <t>Lyria</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Shubin Processing Facility SPMC-1</t>
+          <t>Shubin Processing Facility SPAL-3</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
@@ -7236,12 +7236,12 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Calliope</t>
+          <t>Lyria</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Shubin Processing Facility SPMC-10</t>
+          <t>Shubin Processing Facility SPAL-7</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
@@ -7263,12 +7263,12 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>Calliope</t>
+          <t>Lyria</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Shubin Processing Facility SPMC-11</t>
+          <t>Shubin Processing Facility SPAL-9</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -7295,7 +7295,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Shubin Processing Facility SPMC-14</t>
+          <t>Shubin Processing Facility SPMC-1</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
@@ -7322,7 +7322,7 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Shubin Processing Facility SPMC-3</t>
+          <t>Shubin Processing Facility SPMC-10</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
@@ -7349,7 +7349,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Shubin Processing Facility SPMC-5</t>
+          <t>Shubin Processing Facility SPMC-11</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
@@ -7371,17 +7371,17 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Arial</t>
+          <t>Calliope</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Smokestack</t>
+          <t>Shubin Processing Facility SPMC-14</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>forward_operating_base</t>
+          <t>processing_facility</t>
         </is>
       </c>
       <c r="E256" t="n">
@@ -7393,27 +7393,28 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>Pyro</t>
+          <t>Stanton</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Calliope</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Stanton Jump Point</t>
+          <t>Shubin Processing Facility SPMC-3</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>gateway</t>
+          <t>processing_facility</t>
         </is>
       </c>
       <c r="E257" t="n">
-        <v>1</v>
-      </c>
-      <c r="F257" t="inlineStr">
-        <is>
-          <t>Pyro-Stanton Gate (Pyro side); Pyro Gateway</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F257" t="inlineStr"/>
       <c r="G257" t="inlineStr"/>
     </row>
     <row r="258">
@@ -7424,17 +7425,17 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>Calliope</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Stone's Throw</t>
+          <t>Shubin Processing Facility SPMC-5</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>forward_operating_base</t>
+          <t>processing_facility</t>
         </is>
       </c>
       <c r="E258" t="n">
@@ -7451,17 +7452,17 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Yela</t>
+          <t>Arial</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Talarine Divide Aid Shelter</t>
+          <t>Smokestack</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>shelter</t>
+          <t>forward_operating_base</t>
         </is>
       </c>
       <c r="E259" t="n">
@@ -7473,28 +7474,27 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>Stanton</t>
-        </is>
-      </c>
-      <c r="B260" t="inlineStr">
-        <is>
-          <t>Daymar</t>
+          <t>Pyro</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Tamdon Plains</t>
+          <t>Stanton Jump Point</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>shelter</t>
+          <t>gateway</t>
         </is>
       </c>
       <c r="E260" t="n">
-        <v>0</v>
-      </c>
-      <c r="F260" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Pyro-Stanton Gate (Pyro side); Pyro Gateway</t>
+        </is>
+      </c>
       <c r="G260" t="inlineStr"/>
     </row>
     <row r="261">
@@ -7505,17 +7505,17 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>Cellin</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Tavan</t>
+          <t>Stone's Throw</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>forward_operating_base</t>
         </is>
       </c>
       <c r="E261" t="n">
@@ -7532,17 +7532,17 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>Yela</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Terra Mills HydroFarm</t>
+          <t>Talarine Divide Aid Shelter</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>farm</t>
+          <t>shelter</t>
         </is>
       </c>
       <c r="E262" t="n">
@@ -7564,12 +7564,12 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Thaquray</t>
+          <t>Tamdon Plains</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>shelter</t>
         </is>
       </c>
       <c r="E263" t="n">
@@ -7586,17 +7586,17 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Arial</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>The Dregs</t>
+          <t>Tavan</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>forward_operating_base</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E264" t="n">
@@ -7613,17 +7613,17 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>Crusader</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>The Garden</t>
+          <t>Teasa Spaceport</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>underground_bunker</t>
+          <t>spaceport</t>
         </is>
       </c>
       <c r="E265" t="n">
@@ -7640,17 +7640,17 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>Cellin</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>The Grove</t>
+          <t>Terra Mills HydroFarm</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>forward_operating_base</t>
+          <t>farm</t>
         </is>
       </c>
       <c r="E266" t="n">
@@ -7667,17 +7667,17 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>The Hollows</t>
+          <t>Thaquray</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>forward_operating_base</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E267" t="n">
@@ -7694,17 +7694,17 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Euterpe</t>
+          <t>Arial</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>The Icebreaker</t>
+          <t>The Dregs</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>racetrack</t>
+          <t>forward_operating_base</t>
         </is>
       </c>
       <c r="E268" t="n">
@@ -7721,17 +7721,17 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Ita</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>The Shades</t>
+          <t>The Garden</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>forward_operating_base</t>
+          <t>underground_bunker</t>
         </is>
       </c>
       <c r="E269" t="n">
@@ -7748,12 +7748,12 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Ita</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Thimblerig</t>
+          <t>The Grove</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
@@ -7775,17 +7775,17 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>Cellin</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>TPF</t>
+          <t>The Hollows</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>underground_bunker</t>
+          <t>forward_operating_base</t>
         </is>
       </c>
       <c r="E271" t="n">
@@ -7802,17 +7802,17 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Cellin</t>
+          <t>Euterpe</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Tram &amp; Myers Mining</t>
+          <t>The Icebreaker</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>outpost</t>
+          <t>racetrack</t>
         </is>
       </c>
       <c r="E272" t="n">
@@ -7829,12 +7829,12 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>Ita</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Trilo</t>
+          <t>The Shades</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
@@ -7856,17 +7856,17 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Yela</t>
+          <t>Ita</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Triolet</t>
+          <t>Thimblerig</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>forward_operating_base</t>
         </is>
       </c>
       <c r="E274" t="n">
@@ -7888,12 +7888,12 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>UEES Flyssa</t>
+          <t>TPF</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>wreck_site</t>
+          <t>underground_bunker</t>
         </is>
       </c>
       <c r="E275" t="n">
@@ -7910,17 +7910,17 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>Cellin</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Ulaga</t>
+          <t>Tram &amp; Myers Mining</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>outpost</t>
         </is>
       </c>
       <c r="E276" t="n">
@@ -7937,17 +7937,17 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Yela</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>Utopia</t>
+          <t>Trilo</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>underground_bunker</t>
+          <t>forward_operating_base</t>
         </is>
       </c>
       <c r="E277" t="n">
@@ -7964,17 +7964,17 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>Yela</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Vivere OLP</t>
+          <t>Triolet</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>orbital_laser_platform</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E278" t="n">
@@ -7991,17 +7991,17 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Vivere PAF-I</t>
+          <t>UEES Flyssa</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>planetary_alignment_facility</t>
+          <t>wreck_site</t>
         </is>
       </c>
       <c r="E279" t="n">
@@ -8018,17 +8018,17 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Vivere PAF-II</t>
+          <t>Ulaga</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>planetary_alignment_facility</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E280" t="n">
@@ -8045,17 +8045,17 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>Yela</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Vivere PAF-III</t>
+          <t>Utopia</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>planetary_alignment_facility</t>
+          <t>underground_bunker</t>
         </is>
       </c>
       <c r="E281" t="n">
@@ -8072,17 +8072,17 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>Wailing rock</t>
+          <t>Vivere OLP</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>forward_operating_base</t>
+          <t>orbital_laser_platform</t>
         </is>
       </c>
       <c r="E282" t="n">
@@ -8099,17 +8099,17 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Yela</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Walvis</t>
+          <t>Vivere PAF-I</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>planetary_alignment_facility</t>
         </is>
       </c>
       <c r="E283" t="n">
@@ -8126,17 +8126,17 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Yela</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Wan</t>
+          <t>Vivere PAF-II</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>planetary_alignment_facility</t>
         </is>
       </c>
       <c r="E284" t="n">
@@ -8153,17 +8153,17 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>Weeping Cove</t>
+          <t>Vivere PAF-III</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>settlement</t>
+          <t>planetary_alignment_facility</t>
         </is>
       </c>
       <c r="E285" t="n">
@@ -8185,12 +8185,12 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Whistlers Crypt</t>
+          <t>Wailing rock</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>settlement</t>
+          <t>forward_operating_base</t>
         </is>
       </c>
       <c r="E286" t="n">
@@ -8207,27 +8207,23 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>ARC-L1</t>
+          <t>Yela</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>Wide Forest</t>
+          <t>Walvis</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>lagrange</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E287" t="n">
         <v>0</v>
       </c>
-      <c r="F287" t="inlineStr">
-        <is>
-          <t>ARC-L1 Wide Forest Station; Wild Forest</t>
-        </is>
-      </c>
+      <c r="F287" t="inlineStr"/>
       <c r="G287" t="inlineStr"/>
     </row>
     <row r="288">
@@ -8238,17 +8234,17 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>Yela</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>Wolf Point</t>
+          <t>Wan</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>shelter</t>
+          <t>security_post</t>
         </is>
       </c>
       <c r="E288" t="n">
@@ -8265,17 +8261,17 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Daymar</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Yadar Valley</t>
+          <t>Weeping Cove</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>racetrack</t>
+          <t>settlement</t>
         </is>
       </c>
       <c r="E289" t="n">
@@ -8297,12 +8293,12 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>Yafa</t>
+          <t>Whistlers Crypt</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>security_post</t>
+          <t>settlement</t>
         </is>
       </c>
       <c r="E290" t="n">
@@ -8319,12 +8315,12 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>HUR-L4</t>
+          <t>ARC-L1</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>Yellow Core</t>
+          <t>Wide Forest</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
@@ -8337,7 +8333,7 @@
       </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t>Yellow Core Station</t>
+          <t>ARC-L1 Wide Forest Station; Wild Forest</t>
         </is>
       </c>
       <c r="G291" t="inlineStr"/>
@@ -8350,17 +8346,17 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>Daymar</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Zephyr</t>
+          <t>Wolf Point</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>settlement</t>
+          <t>shelter</t>
         </is>
       </c>
       <c r="E292" t="n">
@@ -8368,6 +8364,118 @@
       </c>
       <c r="F292" t="inlineStr"/>
       <c r="G292" t="inlineStr"/>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>Stanton</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Daymar</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Yadar Valley</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>racetrack</t>
+        </is>
+      </c>
+      <c r="E293" t="n">
+        <v>0</v>
+      </c>
+      <c r="F293" t="inlineStr"/>
+      <c r="G293" t="inlineStr"/>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>Stanton</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Daymar</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Yafa</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>security_post</t>
+        </is>
+      </c>
+      <c r="E294" t="n">
+        <v>0</v>
+      </c>
+      <c r="F294" t="inlineStr"/>
+      <c r="G294" t="inlineStr"/>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Stanton</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>HUR-L4</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Yellow Core</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>lagrange</t>
+        </is>
+      </c>
+      <c r="E295" t="n">
+        <v>0</v>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>Yellow Core Station</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr"/>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>Stanton</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Hurston</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Zephyr</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>settlement</t>
+        </is>
+      </c>
+      <c r="E296" t="n">
+        <v>0</v>
+      </c>
+      <c r="F296" t="inlineStr"/>
+      <c r="G296" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update spaceport locations per crew matching
Sets each spaceport's parent_body and sort_order to match the city
locations provided: August Dunlow -> Orison (Crusader), Riker
Memorial -> Area18 (ArcCorp), Teasa -> Lorville (Hurston), New
Babbage Interstellar -> New Babbage (microTech). Voice-handoff
spreadsheet regenerated.
</commit_message>
<xml_diff>
--- a/scm_stations_voice_handoff.xlsx
+++ b/scm_stations_voice_handoff.xlsx
@@ -1234,7 +1234,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ArcCorp</t>
+          <t>Crusader</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Hurston</t>
+          <t>ArcCorp</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -7613,7 +7613,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Crusader</t>
+          <t>Hurston</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">

</xml_diff>